<commit_message>
Fix project save descriptors and window layouts; localize Excel booleans
</commit_message>
<xml_diff>
--- a/python-version/examples/template_definitions/模板定义示例.xlsx
+++ b/python-version/examples/template_definitions/模板定义示例.xlsx
@@ -19,8 +19,8 @@
     <sheet name="模板设置" sheetId="10" state="visible" r:id="rId10"/>
   </sheets>
   <definedNames>
-    <definedName name="_planner_options_1">'_填写选项'!$A$1:$A$10</definedName>
-    <definedName name="_planner_options_2">'_填写选项'!$B$1:$B$4</definedName>
+    <definedName name="_planner_options_1">'_填写选项'!$A$1:$A$9</definedName>
+    <definedName name="_planner_options_2">'_填写选项'!$B$1:$B$2</definedName>
     <definedName name="_planner_options_3">'_填写选项'!$C$1:$C$6</definedName>
     <definedName name="_planner_options_4">'_填写选项'!$D$1:$D$6</definedName>
     <definedName name="_planner_options_5">'_填写选项'!$E$1:$E$4</definedName>
@@ -206,7 +206,7 @@
     </comment>
     <comment ref="C2" authorId="0" shapeId="0">
       <text>
-        <t>选填：下拉选 float 数值 / int 整数 / category 类别 / bool 是否 / text 文字；留空为 float。</t>
+        <t>选填：下拉选数值 / 整数 / 类别 / 是否 / 文字；是否类型的值填是或否。留空为 float（数值）。</t>
       </text>
     </comment>
     <comment ref="D2" authorId="0" shapeId="0">
@@ -241,7 +241,7 @@
     </comment>
     <comment ref="J2" authorId="0" shapeId="0">
       <text>
-        <t>选填：true/是 或 false/否。文字不能作为数值模型输入；事后或未知测量不能作为未来输入。</t>
+        <t>选填：是 或 否。文字不能作为数值模型输入；事后或未知测量不能作为未来输入。</t>
       </text>
     </comment>
     <comment ref="K2" authorId="0" shapeId="0">
@@ -316,7 +316,7 @@
     </comment>
     <comment ref="C2" authorId="0" shapeId="0">
       <text>
-        <t>选填：下拉选 float 数值 / int 整数 / category 类别 / bool 是否 / text 文字；留空为 float。</t>
+        <t>选填：下拉选数值 / 整数 / 类别 / 是否 / 文字；是否类型的值填是或否。留空为 float（数值）。</t>
       </text>
     </comment>
     <comment ref="D2" authorId="0" shapeId="0">
@@ -351,7 +351,7 @@
     </comment>
     <comment ref="J2" authorId="0" shapeId="0">
       <text>
-        <t>选填：true/是 或 false/否。文字不能作为数值模型输入；事后或未知测量不能作为未来输入。</t>
+        <t>选填：是 或 否。文字不能作为数值模型输入；事后或未知测量不能作为未来输入。</t>
       </text>
     </comment>
     <comment ref="K2" authorId="0" shapeId="0">
@@ -426,7 +426,7 @@
     </comment>
     <comment ref="C2" authorId="0" shapeId="0">
       <text>
-        <t>选填：下拉选 float 数值 / int 整数 / category 类别 / bool 是否 / text 文字；留空为 float。</t>
+        <t>选填：下拉选数值 / 整数 / 类别 / 是否 / 文字；是否类型的值填是或否。留空为 float（数值）。</t>
       </text>
     </comment>
     <comment ref="D2" authorId="0" shapeId="0">
@@ -461,7 +461,7 @@
     </comment>
     <comment ref="J2" authorId="0" shapeId="0">
       <text>
-        <t>选填：true/是 或 false/否。文字不能作为数值模型输入；事后或未知测量不能作为未来输入。</t>
+        <t>选填：是 或 否。文字不能作为数值模型输入；事后或未知测量不能作为未来输入。</t>
       </text>
     </comment>
     <comment ref="K2" authorId="0" shapeId="0">
@@ -561,7 +561,7 @@
   <commentList>
     <comment ref="A2" authorId="0" shapeId="0">
       <text>
-        <t>选填：true/是 启用、false/否 不启用；留空默认启用。</t>
+        <t>选填：是 启用、否 不启用；留空默认启用。</t>
       </text>
     </comment>
     <comment ref="B2" authorId="0" shapeId="0">
@@ -681,7 +681,7 @@
     </comment>
     <comment ref="C2" authorId="0" shapeId="0">
       <text>
-        <t>选填：str 文字 / int 整数 / float 数值 / bool 是否 / list 列表 / dict 对象 / null 空值。</t>
+        <t>选填：str 文字 / int 整数 / float 数值 / 是否 / list 列表 / dict 对象 / null 空值。</t>
       </text>
     </comment>
     <comment ref="D2" authorId="0" shapeId="0">
@@ -1054,7 +1054,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>类型填 float/int/category/bool/text，或 数值/整数/类别/是否/文字。单位可自由填写，无量纲填 1。</t>
+          <t>类型可选数值/整数/类别/是否/文字；是否的填写值选是或否。单位可自由填写，无量纲填 1。</t>
         </is>
       </c>
     </row>
@@ -1082,7 +1082,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>开关列填 是/否 或 true/false；文字/类别测量的作为响应填否。</t>
+          <t>开关列只需选 是/否；是否类型的固定值填是或否，离散值可写 ["是","否"]。文字/类别测量的作为响应填否。</t>
         </is>
       </c>
     </row>
@@ -1175,7 +1175,7 @@
       </c>
       <c r="C1" s="2" t="inlineStr">
         <is>
-          <t>选填：str 文字 / int 整数 / float 数值 / bool 是否 / list 列表 / dict 对象 / null 空值。</t>
+          <t>选填：str 文字 / int 整数 / float 数值 / 是否 / list 列表 / dict 对象 / null 空值。</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
@@ -1427,7 +1427,7 @@
       </c>
       <c r="C1" s="2" t="inlineStr">
         <is>
-          <t>选填：下拉选 float 数值 / int 整数 / category 类别 / bool 是否 / text 文字；留空为 float。</t>
+          <t>选填：下拉选数值 / 整数 / 类别 / 是否 / 文字；是否类型的值填是或否。留空为 float（数值）。</t>
         </is>
       </c>
       <c r="D1" s="2" t="inlineStr">
@@ -1462,7 +1462,7 @@
       </c>
       <c r="J1" s="2" t="inlineStr">
         <is>
-          <t>选填：true/是 或 false/否。文字不能作为数值模型输入；事后或未知测量不能作为未来输入。</t>
+          <t>选填：是 或 否。文字不能作为数值模型输入；事后或未知测量不能作为未来输入。</t>
         </is>
       </c>
       <c r="K1" s="2" t="inlineStr">
@@ -1652,7 +1652,7 @@
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>true</t>
+          <t>是</t>
         </is>
       </c>
       <c r="P3" t="inlineStr">
@@ -1694,14 +1694,14 @@
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>false</t>
+          <t>否</t>
         </is>
       </c>
     </row>
   </sheetData>
   <autoFilter ref="A2:T4"/>
   <dataValidations count="12">
-    <dataValidation sqref="C3:C10002" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="填写内容不符合要求" error="请按列名上方说明填写。复制粘贴后仍需通过软件导入校验。" promptTitle="填写说明" prompt="选填：下拉选 float 数值 / int 整数 / category 类别 / bool 是否 / text 文字；留空为 float。" type="list" errorStyle="stop">
+    <dataValidation sqref="C3:C10002" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="填写内容不符合要求" error="请按列名上方说明填写。复制粘贴后仍需通过软件导入校验。" promptTitle="填写说明" prompt="选填：下拉选数值 / 整数 / 类别 / 是否 / 文字；是否类型的值填是或否。留空为 float（数值）。" type="list" errorStyle="stop">
       <formula1>=_planner_options_1</formula1>
     </dataValidation>
     <dataValidation sqref="F3:F10002" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="填写内容不符合要求" error="请按列名上方说明填写。复制粘贴后仍需通过软件导入校验。" promptTitle="填写说明" prompt="条件必填：用范围定义数值输入时，下限和上限都要填，且下限 &lt; 上限。范围、离散值、固定值三选一。" type="custom" errorStyle="stop">
@@ -1710,7 +1710,7 @@
     <dataValidation sqref="G3:G10002" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="填写内容不符合要求" error="请按列名上方说明填写。复制粘贴后仍需通过软件导入校验。" promptTitle="填写说明" prompt="条件必填：范围输入的上限；必须大于下限。无范围时留空。" type="custom" errorStyle="stop">
       <formula1>OR(G3="",AND(ISNUMBER(G3)))</formula1>
     </dataValidation>
-    <dataValidation sqref="J3:J10002" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="填写内容不符合要求" error="请按列名上方说明填写。复制粘贴后仍需通过软件导入校验。" promptTitle="填写说明" prompt="选填：true/是 或 false/否。文字不能作为数值模型输入；事后或未知测量不能作为未来输入。" type="list" errorStyle="stop">
+    <dataValidation sqref="J3:J10002" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="填写内容不符合要求" error="请按列名上方说明填写。复制粘贴后仍需通过软件导入校验。" promptTitle="填写说明" prompt="选填：是 或 否。文字不能作为数值模型输入；事后或未知测量不能作为未来输入。" type="list" errorStyle="stop">
       <formula1>=_planner_options_2</formula1>
     </dataValidation>
     <dataValidation sqref="K3:K10002" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="填写内容不符合要求" error="请按列名上方说明填写。复制粘贴后仍需通过软件导入校验。" promptTitle="填写说明" prompt="选填：作为响应？原始测量/派生指标的数值字段手写留空默认是；文字/类别不作数值响应。" type="list" errorStyle="stop">
@@ -1749,7 +1749,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L10"/>
+  <dimension ref="A1:L9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1760,7 +1760,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>true</t>
+          <t>是</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
@@ -1822,7 +1822,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>false</t>
+          <t>否</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -1882,11 +1882,6 @@
           <t>category</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>是</t>
-        </is>
-      </c>
       <c r="C3" t="inlineStr">
         <is>
           <t>unknown</t>
@@ -1936,12 +1931,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>bool</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>否</t>
+          <t>text</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -1971,7 +1961,7 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>bool</t>
+          <t>是否</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
@@ -1983,7 +1973,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>数值</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -2015,7 +2005,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>数值</t>
+          <t>整数</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -2042,7 +2032,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>整数</t>
+          <t>类别</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
@@ -2054,19 +2044,12 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>类别</t>
+          <t>是否</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
-        <is>
-          <t>是否</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
         <is>
           <t>文字</t>
         </is>
@@ -2121,7 +2104,7 @@
       </c>
       <c r="C1" s="2" t="inlineStr">
         <is>
-          <t>选填：下拉选 float 数值 / int 整数 / category 类别 / bool 是否 / text 文字；留空为 float。</t>
+          <t>选填：下拉选数值 / 整数 / 类别 / 是否 / 文字；是否类型的值填是或否。留空为 float（数值）。</t>
         </is>
       </c>
       <c r="D1" s="2" t="inlineStr">
@@ -2156,7 +2139,7 @@
       </c>
       <c r="J1" s="2" t="inlineStr">
         <is>
-          <t>选填：true/是 或 false/否。文字不能作为数值模型输入；事后或未知测量不能作为未来输入。</t>
+          <t>选填：是 或 否。文字不能作为数值模型输入；事后或未知测量不能作为未来输入。</t>
         </is>
       </c>
       <c r="K1" s="2" t="inlineStr">
@@ -2340,12 +2323,12 @@
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>true</t>
+          <t>是</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>true</t>
+          <t>是</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
@@ -2357,7 +2340,7 @@
   </sheetData>
   <autoFilter ref="A2:T3"/>
   <dataValidations count="12">
-    <dataValidation sqref="C3:C10002" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="填写内容不符合要求" error="请按列名上方说明填写。复制粘贴后仍需通过软件导入校验。" promptTitle="填写说明" prompt="选填：下拉选 float 数值 / int 整数 / category 类别 / bool 是否 / text 文字；留空为 float。" type="list" errorStyle="stop">
+    <dataValidation sqref="C3:C10002" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="填写内容不符合要求" error="请按列名上方说明填写。复制粘贴后仍需通过软件导入校验。" promptTitle="填写说明" prompt="选填：下拉选数值 / 整数 / 类别 / 是否 / 文字；是否类型的值填是或否。留空为 float（数值）。" type="list" errorStyle="stop">
       <formula1>=_planner_options_1</formula1>
     </dataValidation>
     <dataValidation sqref="F3:F10002" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="填写内容不符合要求" error="请按列名上方说明填写。复制粘贴后仍需通过软件导入校验。" promptTitle="填写说明" prompt="选填：非输入字段通常留空。范围和执行网格仅用于可控输入；下限/上限若填写须成对。" type="custom" errorStyle="stop">
@@ -2366,7 +2349,7 @@
     <dataValidation sqref="G3:G10002" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="填写内容不符合要求" error="请按列名上方说明填写。复制粘贴后仍需通过软件导入校验。" promptTitle="填写说明" prompt="选填：非输入字段通常留空。范围和执行网格仅用于可控输入；下限/上限若填写须成对。" type="custom" errorStyle="stop">
       <formula1>OR(G3="",AND(ISNUMBER(G3)))</formula1>
     </dataValidation>
-    <dataValidation sqref="J3:J10002" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="填写内容不符合要求" error="请按列名上方说明填写。复制粘贴后仍需通过软件导入校验。" promptTitle="填写说明" prompt="选填：true/是 或 false/否。文字不能作为数值模型输入；事后或未知测量不能作为未来输入。" type="list" errorStyle="stop">
+    <dataValidation sqref="J3:J10002" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="填写内容不符合要求" error="请按列名上方说明填写。复制粘贴后仍需通过软件导入校验。" promptTitle="填写说明" prompt="选填：是 或 否。文字不能作为数值模型输入；事后或未知测量不能作为未来输入。" type="list" errorStyle="stop">
       <formula1>=_planner_options_2</formula1>
     </dataValidation>
     <dataValidation sqref="K3:K10002" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="填写内容不符合要求" error="请按列名上方说明填写。复制粘贴后仍需通过软件导入校验。" promptTitle="填写说明" prompt="选填：作为响应？原始测量/派生指标的数值字段手写留空默认是；文字/类别不作数值响应。" type="list" errorStyle="stop">
@@ -2443,7 +2426,7 @@
       </c>
       <c r="C1" s="2" t="inlineStr">
         <is>
-          <t>选填：下拉选 float 数值 / int 整数 / category 类别 / bool 是否 / text 文字；留空为 float。</t>
+          <t>选填：下拉选数值 / 整数 / 类别 / 是否 / 文字；是否类型的值填是或否。留空为 float（数值）。</t>
         </is>
       </c>
       <c r="D1" s="2" t="inlineStr">
@@ -2478,7 +2461,7 @@
       </c>
       <c r="J1" s="2" t="inlineStr">
         <is>
-          <t>选填：true/是 或 false/否。文字不能作为数值模型输入；事后或未知测量不能作为未来输入。</t>
+          <t>选填：是 或 否。文字不能作为数值模型输入；事后或未知测量不能作为未来输入。</t>
         </is>
       </c>
       <c r="K1" s="2" t="inlineStr">
@@ -2657,12 +2640,12 @@
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>true</t>
+          <t>是</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>false</t>
+          <t>否</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
@@ -2674,7 +2657,7 @@
   </sheetData>
   <autoFilter ref="A2:T3"/>
   <dataValidations count="12">
-    <dataValidation sqref="C3:C10002" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="填写内容不符合要求" error="请按列名上方说明填写。复制粘贴后仍需通过软件导入校验。" promptTitle="填写说明" prompt="选填：下拉选 float 数值 / int 整数 / category 类别 / bool 是否 / text 文字；留空为 float。" type="list" errorStyle="stop">
+    <dataValidation sqref="C3:C10002" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="填写内容不符合要求" error="请按列名上方说明填写。复制粘贴后仍需通过软件导入校验。" promptTitle="填写说明" prompt="选填：下拉选数值 / 整数 / 类别 / 是否 / 文字；是否类型的值填是或否。留空为 float（数值）。" type="list" errorStyle="stop">
       <formula1>=_planner_options_1</formula1>
     </dataValidation>
     <dataValidation sqref="F3:F10002" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="填写内容不符合要求" error="请按列名上方说明填写。复制粘贴后仍需通过软件导入校验。" promptTitle="填写说明" prompt="选填：非输入字段通常留空。范围和执行网格仅用于可控输入；下限/上限若填写须成对。" type="custom" errorStyle="stop">
@@ -2683,7 +2666,7 @@
     <dataValidation sqref="G3:G10002" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="填写内容不符合要求" error="请按列名上方说明填写。复制粘贴后仍需通过软件导入校验。" promptTitle="填写说明" prompt="选填：非输入字段通常留空。范围和执行网格仅用于可控输入；下限/上限若填写须成对。" type="custom" errorStyle="stop">
       <formula1>OR(G3="",AND(ISNUMBER(G3)))</formula1>
     </dataValidation>
-    <dataValidation sqref="J3:J10002" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="填写内容不符合要求" error="请按列名上方说明填写。复制粘贴后仍需通过软件导入校验。" promptTitle="填写说明" prompt="选填：true/是 或 false/否。文字不能作为数值模型输入；事后或未知测量不能作为未来输入。" type="list" errorStyle="stop">
+    <dataValidation sqref="J3:J10002" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="填写内容不符合要求" error="请按列名上方说明填写。复制粘贴后仍需通过软件导入校验。" promptTitle="填写说明" prompt="选填：是 或 否。文字不能作为数值模型输入；事后或未知测量不能作为未来输入。" type="list" errorStyle="stop">
       <formula1>=_planner_options_2</formula1>
     </dataValidation>
     <dataValidation sqref="K3:K10002" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="填写内容不符合要求" error="请按列名上方说明填写。复制粘贴后仍需通过软件导入校验。" promptTitle="填写说明" prompt="选填：作为响应？原始测量/派生指标的数值字段手写留空默认是；文字/类别不作数值响应。" type="list" errorStyle="stop">
@@ -2843,7 +2826,7 @@
     <row r="1" ht="110" customHeight="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>【填写提示】选填：true/是 启用、false/否 不启用；留空默认启用。</t>
+          <t>【填写提示】选填：是 启用、否 不启用；留空默认启用。</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
@@ -2927,7 +2910,7 @@
   </sheetData>
   <autoFilter ref="A2:H2"/>
   <dataValidations count="4">
-    <dataValidation sqref="A3:A10002" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="填写内容不符合要求" error="请按列名上方说明填写。复制粘贴后仍需通过软件导入校验。" promptTitle="填写说明" prompt="选填：true/是 启用、false/否 不启用；留空默认启用。" type="list" errorStyle="stop">
+    <dataValidation sqref="A3:A10002" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="填写内容不符合要求" error="请按列名上方说明填写。复制粘贴后仍需通过软件导入校验。" promptTitle="填写说明" prompt="选填：是 启用、否 不启用；留空默认启用。" type="list" errorStyle="stop">
       <formula1>=_planner_options_2</formula1>
     </dataValidation>
     <dataValidation sqref="D3:D10002" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="填写内容不符合要求" error="请按列名上方说明填写。复制粘贴后仍需通过软件导入校验。" promptTitle="填写说明" prompt="启用时必填：independent 独立、linear 线性、proportional 比例、monotonic 单调、weak 弱先验。" type="list" errorStyle="stop">

</xml_diff>